<commit_message>
Correction slicing de clinicalDocument section 9c207da324e6c5249f08e58799b5162fd7c38126
</commit_message>
<xml_diff>
--- a/correctionSlicing/ig/StructureDefinition-fr-cda-clinical-document-ips.xlsx
+++ b/correctionSlicing/ig/StructureDefinition-fr-cda-clinical-document-ips.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-06T09:09:22+00:00</t>
+    <t>2026-10-06T09:25:27+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -952,7 +952,7 @@
     <t>Used to represent other participants not explicitly mentioned by other classes, that were somehow involved in the documented acts.</t>
   </si>
   <si>
-    <t xml:space="preserve">value:url}
+    <t xml:space="preserve">value:functionCode.code}
 </t>
   </si>
   <si>
@@ -3302,7 +3302,7 @@
     <col min="25" max="25" width="18.49609375" customWidth="true" bestFit="true"/>
     <col min="26" max="26" width="89.12890625" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
+    <col min="28" max="28" width="21.453125" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>
     <col min="30" max="30" width="14.7578125" customWidth="true" bestFit="true"/>
     <col min="31" max="31" width="12.359375" customWidth="true" bestFit="true" hidden="true"/>

</xml_diff>

<commit_message>
Correction slicing de clinicalDocument section 4a196a47b972e96017c9b90f0ab2155665277c85
</commit_message>
<xml_diff>
--- a/correctionSlicing/ig/StructureDefinition-fr-cda-clinical-document-ips.xlsx
+++ b/correctionSlicing/ig/StructureDefinition-fr-cda-clinical-document-ips.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17518" uniqueCount="965">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17114" uniqueCount="951">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-06T09:25:27+00:00</t>
+    <t>2026-10-06T09:30:18+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2837,48 +2837,6 @@
   <si>
     <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/Section {https://interop.esante.gouv.fr/ig/cda/document-core/StructureDefinition/fr-cda-plan-de-soins|0.1.0}
 </t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees</t>
-  </si>
-  <si>
-    <t>sectionDirectivesAnticipees</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.nullFlavor</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.realmCode</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.typeId</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.typeId.nullFlavor</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.typeId.assigningAuthorityName</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.typeId.displayable</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.typeId.root</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.typeId.extension</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.templateId</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.typeCode</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.contextConductionInd</t>
-  </si>
-  <si>
-    <t>ClinicalDocument.component.structuredBody.component:sectionDirectivesAnticipees.section</t>
   </si>
   <si>
     <t>ClinicalDocument.component.structuredBody.component:sectionResultats</t>
@@ -3272,7 +3230,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK558"/>
+  <dimension ref="A1:AK545"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="110.40234375" customWidth="true" bestFit="true"/>
@@ -57336,7 +57294,7 @@
         <v>75</v>
       </c>
       <c r="K532" t="s" s="2">
-        <v>679</v>
+        <v>935</v>
       </c>
       <c r="L532" s="2"/>
       <c r="M532" s="2"/>
@@ -57409,13 +57367,13 @@
     </row>
     <row r="533">
       <c r="A533" t="s" s="2">
-        <v>935</v>
+        <v>936</v>
       </c>
       <c r="B533" t="s" s="2">
         <v>659</v>
       </c>
       <c r="C533" t="s" s="2">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="D533" t="s" s="2">
         <v>75</v>
@@ -57510,7 +57468,7 @@
     </row>
     <row r="534">
       <c r="A534" t="s" s="2">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="B534" t="s" s="2">
         <v>665</v>
@@ -57611,7 +57569,7 @@
     </row>
     <row r="535">
       <c r="A535" t="s" s="2">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="B535" t="s" s="2">
         <v>666</v>
@@ -57712,7 +57670,7 @@
     </row>
     <row r="536">
       <c r="A536" t="s" s="2">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="B536" t="s" s="2">
         <v>667</v>
@@ -57813,7 +57771,7 @@
     </row>
     <row r="537">
       <c r="A537" t="s" s="2">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="B537" t="s" s="2">
         <v>668</v>
@@ -57914,7 +57872,7 @@
     </row>
     <row r="538">
       <c r="A538" t="s" s="2">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="B538" t="s" s="2">
         <v>669</v>
@@ -58017,7 +57975,7 @@
     </row>
     <row r="539">
       <c r="A539" t="s" s="2">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="B539" t="s" s="2">
         <v>670</v>
@@ -58120,7 +58078,7 @@
     </row>
     <row r="540">
       <c r="A540" t="s" s="2">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="B540" t="s" s="2">
         <v>671</v>
@@ -58223,7 +58181,7 @@
     </row>
     <row r="541">
       <c r="A541" t="s" s="2">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="B541" t="s" s="2">
         <v>672</v>
@@ -58326,7 +58284,7 @@
     </row>
     <row r="542">
       <c r="A542" t="s" s="2">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="B542" t="s" s="2">
         <v>673</v>
@@ -58427,7 +58385,7 @@
     </row>
     <row r="543">
       <c r="A543" t="s" s="2">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="B543" t="s" s="2">
         <v>674</v>
@@ -58526,7 +58484,7 @@
     </row>
     <row r="544">
       <c r="A544" t="s" s="2">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="B544" t="s" s="2">
         <v>676</v>
@@ -58625,7 +58583,7 @@
     </row>
     <row r="545">
       <c r="A545" t="s" s="2">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="B545" t="s" s="2">
         <v>678</v>
@@ -58651,7 +58609,7 @@
         <v>75</v>
       </c>
       <c r="K545" t="s" s="2">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="L545" s="2"/>
       <c r="M545" s="2"/>
@@ -58722,1321 +58680,6 @@
         <v>75</v>
       </c>
     </row>
-    <row r="546">
-      <c r="A546" t="s" s="2">
-        <v>950</v>
-      </c>
-      <c r="B546" t="s" s="2">
-        <v>659</v>
-      </c>
-      <c r="C546" t="s" s="2">
-        <v>951</v>
-      </c>
-      <c r="D546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E546" s="2"/>
-      <c r="F546" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G546" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K546" t="s" s="2">
-        <v>661</v>
-      </c>
-      <c r="L546" s="2"/>
-      <c r="M546" s="2"/>
-      <c r="N546" s="2"/>
-      <c r="O546" s="2"/>
-      <c r="P546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q546" s="2"/>
-      <c r="R546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF546" t="s" s="2">
-        <v>664</v>
-      </c>
-      <c r="AG546" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH546" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AI546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ546" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK546" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="547">
-      <c r="A547" t="s" s="2">
-        <v>952</v>
-      </c>
-      <c r="B547" t="s" s="2">
-        <v>665</v>
-      </c>
-      <c r="C547" s="2"/>
-      <c r="D547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E547" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="F547" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G547" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K547" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="L547" s="2"/>
-      <c r="M547" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="N547" s="2"/>
-      <c r="O547" s="2"/>
-      <c r="P547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q547" s="2"/>
-      <c r="R547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X547" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="Y547" s="2"/>
-      <c r="Z547" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AA547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF547" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AG547" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH547" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ547" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK547" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="548">
-      <c r="A548" t="s" s="2">
-        <v>953</v>
-      </c>
-      <c r="B548" t="s" s="2">
-        <v>666</v>
-      </c>
-      <c r="C548" s="2"/>
-      <c r="D548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E548" s="2"/>
-      <c r="F548" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G548" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="H548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K548" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="L548" s="2"/>
-      <c r="M548" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="N548" s="2"/>
-      <c r="O548" s="2"/>
-      <c r="P548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q548" s="2"/>
-      <c r="R548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF548" t="s" s="2">
-        <v>310</v>
-      </c>
-      <c r="AG548" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH548" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AI548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ548" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK548" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="549">
-      <c r="A549" t="s" s="2">
-        <v>954</v>
-      </c>
-      <c r="B549" t="s" s="2">
-        <v>667</v>
-      </c>
-      <c r="C549" s="2"/>
-      <c r="D549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E549" s="2"/>
-      <c r="F549" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G549" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K549" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="L549" s="2"/>
-      <c r="M549" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="N549" s="2"/>
-      <c r="O549" s="2"/>
-      <c r="P549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q549" s="2"/>
-      <c r="R549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF549" t="s" s="2">
-        <v>314</v>
-      </c>
-      <c r="AG549" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH549" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI549" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ549" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="AK549" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="550">
-      <c r="A550" t="s" s="2">
-        <v>955</v>
-      </c>
-      <c r="B550" t="s" s="2">
-        <v>668</v>
-      </c>
-      <c r="C550" s="2"/>
-      <c r="D550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E550" t="s" s="2">
-        <v>86</v>
-      </c>
-      <c r="F550" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G550" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K550" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="L550" s="2"/>
-      <c r="M550" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="N550" s="2"/>
-      <c r="O550" s="2"/>
-      <c r="P550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q550" s="2"/>
-      <c r="R550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X550" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="Y550" s="2"/>
-      <c r="Z550" t="s" s="2">
-        <v>90</v>
-      </c>
-      <c r="AA550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF550" t="s" s="2">
-        <v>91</v>
-      </c>
-      <c r="AG550" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH550" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ550" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK550" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="551">
-      <c r="A551" t="s" s="2">
-        <v>956</v>
-      </c>
-      <c r="B551" t="s" s="2">
-        <v>669</v>
-      </c>
-      <c r="C551" s="2"/>
-      <c r="D551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E551" t="s" s="2">
-        <v>110</v>
-      </c>
-      <c r="F551" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G551" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K551" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="L551" s="2"/>
-      <c r="M551" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="N551" s="2"/>
-      <c r="O551" s="2"/>
-      <c r="P551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q551" s="2"/>
-      <c r="R551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF551" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="AG551" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH551" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ551" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK551" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="552">
-      <c r="A552" t="s" s="2">
-        <v>957</v>
-      </c>
-      <c r="B552" t="s" s="2">
-        <v>670</v>
-      </c>
-      <c r="C552" s="2"/>
-      <c r="D552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E552" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="F552" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G552" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K552" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="L552" s="2"/>
-      <c r="M552" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="N552" s="2"/>
-      <c r="O552" s="2"/>
-      <c r="P552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q552" s="2"/>
-      <c r="R552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF552" t="s" s="2">
-        <v>118</v>
-      </c>
-      <c r="AG552" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH552" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ552" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK552" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="553">
-      <c r="A553" t="s" s="2">
-        <v>958</v>
-      </c>
-      <c r="B553" t="s" s="2">
-        <v>671</v>
-      </c>
-      <c r="C553" s="2"/>
-      <c r="D553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E553" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="F553" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G553" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K553" t="s" s="2">
-        <v>121</v>
-      </c>
-      <c r="L553" s="2"/>
-      <c r="M553" t="s" s="2">
-        <v>122</v>
-      </c>
-      <c r="N553" s="2"/>
-      <c r="O553" s="2"/>
-      <c r="P553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q553" s="2"/>
-      <c r="R553" t="s" s="2">
-        <v>123</v>
-      </c>
-      <c r="S553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF553" t="s" s="2">
-        <v>124</v>
-      </c>
-      <c r="AG553" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH553" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ553" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK553" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="554">
-      <c r="A554" t="s" s="2">
-        <v>959</v>
-      </c>
-      <c r="B554" t="s" s="2">
-        <v>672</v>
-      </c>
-      <c r="C554" s="2"/>
-      <c r="D554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E554" t="s" s="2">
-        <v>126</v>
-      </c>
-      <c r="F554" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G554" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K554" t="s" s="2">
-        <v>111</v>
-      </c>
-      <c r="L554" s="2"/>
-      <c r="M554" t="s" s="2">
-        <v>127</v>
-      </c>
-      <c r="N554" s="2"/>
-      <c r="O554" s="2"/>
-      <c r="P554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q554" s="2"/>
-      <c r="R554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF554" t="s" s="2">
-        <v>129</v>
-      </c>
-      <c r="AG554" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH554" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ554" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK554" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="555">
-      <c r="A555" t="s" s="2">
-        <v>960</v>
-      </c>
-      <c r="B555" t="s" s="2">
-        <v>673</v>
-      </c>
-      <c r="C555" s="2"/>
-      <c r="D555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E555" s="2"/>
-      <c r="F555" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G555" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="H555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K555" t="s" s="2">
-        <v>104</v>
-      </c>
-      <c r="L555" s="2"/>
-      <c r="M555" t="s" s="2">
-        <v>133</v>
-      </c>
-      <c r="N555" s="2"/>
-      <c r="O555" s="2"/>
-      <c r="P555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q555" s="2"/>
-      <c r="R555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF555" t="s" s="2">
-        <v>327</v>
-      </c>
-      <c r="AG555" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH555" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="AI555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ555" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK555" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="556">
-      <c r="A556" t="s" s="2">
-        <v>961</v>
-      </c>
-      <c r="B556" t="s" s="2">
-        <v>674</v>
-      </c>
-      <c r="C556" s="2"/>
-      <c r="D556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E556" s="2"/>
-      <c r="F556" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G556" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K556" t="s" s="2">
-        <v>87</v>
-      </c>
-      <c r="L556" s="2"/>
-      <c r="M556" s="2"/>
-      <c r="N556" s="2"/>
-      <c r="O556" s="2"/>
-      <c r="P556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q556" s="2"/>
-      <c r="R556" t="s" s="2">
-        <v>626</v>
-      </c>
-      <c r="S556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF556" t="s" s="2">
-        <v>675</v>
-      </c>
-      <c r="AG556" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH556" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ556" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK556" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="557">
-      <c r="A557" t="s" s="2">
-        <v>962</v>
-      </c>
-      <c r="B557" t="s" s="2">
-        <v>676</v>
-      </c>
-      <c r="C557" s="2"/>
-      <c r="D557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E557" s="2"/>
-      <c r="F557" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G557" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K557" t="s" s="2">
-        <v>116</v>
-      </c>
-      <c r="L557" s="2"/>
-      <c r="M557" s="2"/>
-      <c r="N557" s="2"/>
-      <c r="O557" s="2"/>
-      <c r="P557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q557" s="2"/>
-      <c r="R557" t="s" s="2">
-        <v>630</v>
-      </c>
-      <c r="S557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF557" t="s" s="2">
-        <v>677</v>
-      </c>
-      <c r="AG557" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH557" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ557" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK557" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="558">
-      <c r="A558" t="s" s="2">
-        <v>963</v>
-      </c>
-      <c r="B558" t="s" s="2">
-        <v>678</v>
-      </c>
-      <c r="C558" s="2"/>
-      <c r="D558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="E558" s="2"/>
-      <c r="F558" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="G558" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="I558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="J558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="K558" t="s" s="2">
-        <v>964</v>
-      </c>
-      <c r="L558" s="2"/>
-      <c r="M558" s="2"/>
-      <c r="N558" s="2"/>
-      <c r="O558" s="2"/>
-      <c r="P558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Q558" s="2"/>
-      <c r="R558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="S558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="T558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="U558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="V558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="W558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="X558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Y558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="Z558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AA558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AB558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AC558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AD558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AE558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AF558" t="s" s="2">
-        <v>680</v>
-      </c>
-      <c r="AG558" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AH558" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AJ558" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AK558" t="s" s="2">
-        <v>75</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Correction slicing participant IPS et corrections de l'exemple CDA
- FRCDAClinicalDocumentIPS : discriminateurs functionCode.code et typeCode
  sur participant (conflit contactEHPAD / autreCorrespondant)
- Binary-patient-summary.xml : libellé « Sœur », références du narratif
  (#med-03, #resultat-imagerie-02*, ID resultat-02), displayName de la section d6d5d96fccd3800471e1f19ca816fe4d843143c7
</commit_message>
<xml_diff>
--- a/correctionSlicing/ig/StructureDefinition-fr-cda-clinical-document-ips.xlsx
+++ b/correctionSlicing/ig/StructureDefinition-fr-cda-clinical-document-ips.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-10-06T09:30:18+00:00</t>
+    <t>2026-10-09T13:27:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -952,8 +952,8 @@
     <t>Used to represent other participants not explicitly mentioned by other classes, that were somehow involved in the documented acts.</t>
   </si>
   <si>
-    <t xml:space="preserve">value:functionCode.code}
-</t>
+    <t>value:functionCode.code}
+value:typeCode}</t>
   </si>
   <si>
     <t>ClinicalDocument.participant:medecinTraitant</t>

</xml_diff>